<commit_message>
Publicar recursos actualizados de Viko
</commit_message>
<xml_diff>
--- a/Viko/Paladin Spells.xlsx
+++ b/Viko/Paladin Spells.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4604e5eff5508ce9/Desktop/WIZARD SPELLS/Viko/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="182" documentId="8_{969E3AEE-D2B4-4A86-9E37-EFC5ED53D20C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5EE66114-D538-4B8E-875E-A6E2B8F7A5F9}"/>
+  <xr:revisionPtr revIDLastSave="189" documentId="8_{969E3AEE-D2B4-4A86-9E37-EFC5ED53D20C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{948A1172-4BB8-4B71-9E2C-4BF4A3A31229}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{1A773363-9EAE-4410-83FA-4C280E3FC519}"/>
   </bookViews>
@@ -1580,7 +1580,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05DEE858-56F0-465A-9EC7-764476F2B89A}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:M37"/>
+  <dimension ref="A1:M43"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.5546875" style="3"/>
@@ -1635,7 +1635,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="214.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" ht="214.8" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="9">
         <v>1</v>
       </c>
@@ -1674,7 +1674,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="9">
         <v>1</v>
       </c>
@@ -1711,7 +1711,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="9">
         <v>1</v>
       </c>
@@ -1744,7 +1744,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="9">
         <v>1</v>
       </c>
@@ -1777,7 +1777,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="21" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="9">
         <v>1</v>
       </c>
@@ -1810,7 +1810,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="18.600000000000001" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" ht="18.600000000000001" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="9">
         <v>1</v>
       </c>
@@ -1843,7 +1843,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="15.6" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="9">
         <v>1</v>
       </c>
@@ -1876,7 +1876,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="22.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13" ht="22.8" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="9">
         <v>1</v>
       </c>
@@ -1909,7 +1909,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="9">
         <v>1</v>
       </c>
@@ -1942,7 +1942,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="15.6" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="9">
         <v>1</v>
       </c>
@@ -1975,7 +1975,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="21" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" ht="21" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="9">
         <v>1</v>
       </c>
@@ -2006,7 +2006,7 @@
       </c>
       <c r="K12" s="10"/>
     </row>
-    <row r="13" spans="1:13" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" ht="15.6" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="9">
         <v>1</v>
       </c>
@@ -2039,7 +2039,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="9">
         <v>1</v>
       </c>
@@ -2072,7 +2072,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="15.6" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:13" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="9">
         <v>1</v>
       </c>
@@ -2105,7 +2105,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="15.6" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:13" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="9">
         <v>1</v>
       </c>
@@ -2138,7 +2138,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="9">
         <v>1</v>
       </c>
@@ -2171,7 +2171,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="15">
         <v>2</v>
       </c>
@@ -2204,7 +2204,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="22.8" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" ht="22.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="15">
         <v>2</v>
       </c>
@@ -2237,7 +2237,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="22.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" ht="22.8" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="15">
         <v>2</v>
       </c>
@@ -2270,7 +2270,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="22.8" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" ht="22.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="15"/>
       <c r="B21" s="15"/>
       <c r="C21" s="22" t="s">
@@ -2301,7 +2301,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="15">
         <v>2</v>
       </c>
@@ -2334,7 +2334,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" ht="15.6" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="15">
         <v>2</v>
       </c>
@@ -2367,7 +2367,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" ht="24" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="15">
         <v>2</v>
       </c>
@@ -2400,7 +2400,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="27" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" ht="27" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="15">
         <v>2</v>
       </c>
@@ -2433,7 +2433,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="15">
         <v>2</v>
       </c>
@@ -2466,7 +2466,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="15">
         <v>2</v>
       </c>
@@ -2499,7 +2499,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="18" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" ht="18" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="15">
         <v>2</v>
       </c>
@@ -2532,7 +2532,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" ht="15.6" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="15">
         <v>2</v>
       </c>
@@ -2563,7 +2563,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="16" t="s">
         <v>103</v>
       </c>
@@ -2596,7 +2596,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="16" t="s">
         <v>103</v>
       </c>
@@ -2629,7 +2629,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="15.6" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="16" t="s">
         <v>103</v>
       </c>
@@ -2662,7 +2662,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="16" t="s">
         <v>103</v>
       </c>
@@ -2695,7 +2695,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="20.399999999999999" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" ht="20.399999999999999" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="17" t="s">
         <v>107</v>
       </c>
@@ -2728,7 +2728,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:11" ht="30" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="17" t="s">
         <v>107</v>
       </c>
@@ -2761,7 +2761,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" ht="15.6" hidden="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="17" t="s">
         <v>107</v>
       </c>
@@ -2795,11 +2795,29 @@
       </c>
     </row>
     <row r="37" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B43"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K36" xr:uid="{05DEE858-56F0-465A-9EC7-764476F2B89A}">
-    <filterColumn colId="8">
+    <filterColumn colId="2">
       <filters>
-        <filter val="No"/>
+        <filter val="Branding Smite (Castigo marcador)"/>
+        <filter val="Compelled Duel (Duelo Obligado)"/>
+        <filter val="Detect Evil and Good"/>
+        <filter val="Detect Magic"/>
+        <filter val="Detect Poison and Disease"/>
+        <filter val="Divine Favor (Favor Divino)"/>
+        <filter val="Enhance Ability"/>
+        <filter val="Heroism"/>
+        <filter val="Locate Object"/>
+        <filter val="Magic Weapon"/>
+        <filter val="Protection from Evil and Good"/>
+        <filter val="Searing Smite (Castigo Ardiente)"/>
+        <filter val="Shield of Faith (Escudo de Fe)"/>
+        <filter val="Shining Smite (Castigo Luminoso)"/>
+        <filter val="Thunderous Smite (Castigo Atronador)"/>
+        <filter val="Wrathful Smite (Castigo Colérico)"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>